<commit_message>
create synthetich data and evaluate euclidean dist
</commit_message>
<xml_diff>
--- a/Groundtruth/Accuracy.xlsx
+++ b/Groundtruth/Accuracy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\VIS2025\BIoVisChallenges\SSGAT\Groundtruth\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C614BD4B-8C24-4A83-88EC-A60AC7D4E93B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BF646BA-3328-4CE6-B9D2-3ACB5E9BF7B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="984" yWindow="2664" windowWidth="17280" windowHeight="8880" xr2:uid="{DC385397-815F-4A8C-B156-510366D663B0}"/>
+    <workbookView xWindow="30855" yWindow="2835" windowWidth="17280" windowHeight="8880" xr2:uid="{DC385397-815F-4A8C-B156-510366D663B0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -549,10 +549,10 @@
         <v>22</v>
       </c>
       <c r="B3" s="1">
-        <v>0.81</v>
+        <v>0.91</v>
       </c>
       <c r="C3" s="1">
-        <v>0.68069999999999997</v>
+        <v>0.83069999999999999</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1"/>
@@ -573,10 +573,10 @@
         <v>14</v>
       </c>
       <c r="B4" s="1">
-        <v>0.86</v>
+        <v>0.71</v>
       </c>
       <c r="C4" s="1">
-        <v>0.75439999999999996</v>
+        <v>0.5544</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1"/>
@@ -597,10 +597,10 @@
         <v>12</v>
       </c>
       <c r="B5" s="1">
-        <v>0.87</v>
+        <v>0.88</v>
       </c>
       <c r="C5" s="1">
-        <v>0.79239999999999999</v>
+        <v>0.78239999999999998</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
@@ -621,10 +621,10 @@
         <v>11</v>
       </c>
       <c r="B6" s="1">
-        <v>0.84</v>
+        <v>0.92400000000000004</v>
       </c>
       <c r="C6" s="1">
-        <v>0.72409999999999997</v>
+        <v>0.85409999999999997</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1"/>
@@ -645,10 +645,10 @@
         <v>15</v>
       </c>
       <c r="B7" s="1">
-        <v>0.82</v>
+        <v>0.87</v>
       </c>
       <c r="C7" s="1">
-        <v>0.69489999999999996</v>
+        <v>0.77490000000000003</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1"/>
@@ -693,10 +693,10 @@
         <v>20</v>
       </c>
       <c r="B9" s="1">
-        <v>0.8</v>
+        <v>0.81</v>
       </c>
       <c r="C9" s="1">
-        <v>0.65290000000000004</v>
+        <v>0.68289999999999995</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
@@ -717,10 +717,10 @@
         <v>17</v>
       </c>
       <c r="B10" s="1">
-        <v>0.67</v>
+        <v>0.92700000000000005</v>
       </c>
       <c r="C10" s="1">
-        <v>0.59860000000000002</v>
+        <v>0.85160000000000002</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
@@ -741,10 +741,10 @@
         <v>16</v>
       </c>
       <c r="B11" s="1">
-        <v>0.82</v>
+        <v>0.67200000000000004</v>
       </c>
       <c r="C11" s="1">
-        <v>0.75190000000000001</v>
+        <v>0.50190000000000001</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
@@ -765,10 +765,10 @@
         <v>18</v>
       </c>
       <c r="B12" s="1">
-        <v>0.69</v>
+        <v>0.69199999999999995</v>
       </c>
       <c r="C12" s="1">
-        <v>0.61150000000000004</v>
+        <v>0.83150000000000002</v>
       </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
@@ -789,10 +789,10 @@
         <v>0</v>
       </c>
       <c r="B13" s="1">
-        <v>0.71</v>
+        <v>0.83099999999999996</v>
       </c>
       <c r="C13" s="1">
-        <v>0.63849999999999996</v>
+        <v>0.71850000000000003</v>
       </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
@@ -813,10 +813,10 @@
         <v>1</v>
       </c>
       <c r="B14" s="1">
-        <v>0.78</v>
+        <v>0.89100000000000001</v>
       </c>
       <c r="C14" s="1">
-        <v>0.63929999999999998</v>
+        <v>0.81930000000000003</v>
       </c>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
@@ -837,10 +837,10 @@
         <v>2</v>
       </c>
       <c r="B15" s="1">
-        <v>0.81</v>
+        <v>0.79100000000000004</v>
       </c>
       <c r="C15" s="1">
-        <v>0.68069999999999997</v>
+        <v>0.65069999999999995</v>
       </c>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
@@ -861,10 +861,10 @@
         <v>3</v>
       </c>
       <c r="B16" s="1">
-        <v>0.9</v>
+        <v>0.94</v>
       </c>
       <c r="C16" s="1">
-        <v>0.81</v>
+        <v>0.89100000000000001</v>
       </c>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
@@ -885,10 +885,10 @@
         <v>4</v>
       </c>
       <c r="B17" s="1">
-        <v>0.89</v>
+        <v>0.85099999999999998</v>
       </c>
       <c r="C17" s="1">
-        <v>0.80900000000000005</v>
+        <v>0.7409</v>
       </c>
       <c r="D17" s="2"/>
       <c r="E17" s="1"/>

</xml_diff>